<commit_message>
feat(security): SEC-18 — specification_reference as CFTS084-{NRL}, one per line, security_v12
</commit_message>
<xml_diff>
--- a/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
+++ b/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
@@ -8014,7 +8014,47 @@
       </c>
       <c r="N10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-001</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O10" s="81" t="inlineStr">
@@ -8159,7 +8199,47 @@
       </c>
       <c r="N11" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-001</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O11" s="178" t="inlineStr">
@@ -8307,7 +8387,18 @@
       </c>
       <c r="N12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-002</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O12" s="81" t="inlineStr">
@@ -8453,7 +8544,18 @@
       </c>
       <c r="N13" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-002</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O13" s="178" t="inlineStr">
@@ -8601,7 +8703,18 @@
       </c>
       <c r="N14" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-003</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O14" s="81" t="inlineStr">
@@ -8747,7 +8860,18 @@
       </c>
       <c r="N15" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-003</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O15" s="178" t="inlineStr">
@@ -8892,7 +9016,18 @@
       </c>
       <c r="N16" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-004</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O16" s="178" t="inlineStr">
@@ -9036,7 +9171,18 @@
       </c>
       <c r="N17" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-004</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O17" s="81" t="inlineStr">
@@ -9176,7 +9322,18 @@
       </c>
       <c r="N18" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-005</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O18" s="178" t="inlineStr">
@@ -9318,7 +9475,18 @@
       </c>
       <c r="N19" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-005</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O19" s="81" t="inlineStr">
@@ -9458,7 +9626,18 @@
       </c>
       <c r="N20" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-006</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O20" s="81" t="inlineStr">
@@ -9597,7 +9776,18 @@
       </c>
       <c r="N21" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-006</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O21" s="81" t="inlineStr">
@@ -9736,7 +9926,18 @@
       </c>
       <c r="N22" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-006</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O22" s="81" t="inlineStr">
@@ -9875,7 +10076,18 @@
       </c>
       <c r="N23" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-006</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O23" s="81" t="inlineStr">
@@ -10015,7 +10227,39 @@
       </c>
       <c r="N24" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-007</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O24" s="81" t="inlineStr">
@@ -10161,7 +10405,39 @@
       </c>
       <c r="N25" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-007</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O25" s="178" t="inlineStr">
@@ -10308,7 +10584,12 @@
       </c>
       <c r="N26" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-008</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646</t>
         </is>
       </c>
       <c r="O26" s="178" t="inlineStr">
@@ -10454,7 +10735,12 @@
       </c>
       <c r="N27" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-008</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646</t>
         </is>
       </c>
       <c r="O27" s="178" t="inlineStr">
@@ -10598,7 +10884,39 @@
       </c>
       <c r="N28" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-009</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O28" s="81" t="inlineStr">
@@ -10741,7 +11059,39 @@
       </c>
       <c r="N29" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-009</t>
+          <t xml:space="preserve">CFTS084-134408
+CFTS084-134409
+CFTS084-134410
+CFTS084-134411
+CFTS084-134413
+CFTS084-134561
+CFTS084-134562
+CFTS084-134566
+CFTS084-134568
+CFTS084-134644
+CFTS084-134646
+CFTS084-134701
+CFTS084-134702
+CFTS084-134703
+CFTS084-134704
+CFTS084-134705
+CFTS084-134706
+CFTS084-134707
+CFTS084-134711
+CFTS084-134712
+CFTS084-134718
+CFTS084-134724
+CFTS084-134725
+CFTS084-134727
+CFTS084-134728
+CFTS084-134729
+CFTS084-134730
+CFTS084-134731
+CFTS084-134732
+CFTS084-134733
+CFTS084-134734
+CFTS084-134735
+CFTS084-134736</t>
         </is>
       </c>
       <c r="O29" s="178" t="inlineStr">
@@ -10886,7 +11236,18 @@
       </c>
       <c r="N30" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-010</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O30" s="81" t="inlineStr">
@@ -11031,7 +11392,18 @@
       </c>
       <c r="N31" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-011</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O31" s="178" t="inlineStr">
@@ -11174,7 +11546,18 @@
       </c>
       <c r="N32" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-011</t>
+          <t xml:space="preserve">CFTS084-134565
+CFTS084-134566
+CFTS084-134568
+CFTS084-134569
+CFTS084-134570
+CFTS084-134644
+CFTS084-134645
+CFTS084-134646
+CFTS084-134714
+CFTS084-134715
+CFTS084-134716
+CFTS084-134717</t>
         </is>
       </c>
       <c r="O32" s="178" t="inlineStr">

</xml_diff>

<commit_message>
feat(security): SEC-19 — specification_reference numbers switch to Polarion ObjectID, security_v13
</commit_message>
<xml_diff>
--- a/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
+++ b/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
@@ -8014,47 +8014,47 @@
       </c>
       <c r="N10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O10" s="81" t="inlineStr">
@@ -8199,47 +8199,47 @@
       </c>
       <c r="N11" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O11" s="178" t="inlineStr">
@@ -8387,18 +8387,18 @@
       </c>
       <c r="N12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O12" s="81" t="inlineStr">
@@ -8544,18 +8544,18 @@
       </c>
       <c r="N13" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O13" s="178" t="inlineStr">
@@ -8703,18 +8703,18 @@
       </c>
       <c r="N14" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O14" s="81" t="inlineStr">
@@ -8860,18 +8860,18 @@
       </c>
       <c r="N15" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O15" s="178" t="inlineStr">
@@ -9016,18 +9016,18 @@
       </c>
       <c r="N16" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O16" s="178" t="inlineStr">
@@ -9171,18 +9171,18 @@
       </c>
       <c r="N17" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O17" s="81" t="inlineStr">
@@ -9322,18 +9322,18 @@
       </c>
       <c r="N18" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O18" s="178" t="inlineStr">
@@ -9475,18 +9475,18 @@
       </c>
       <c r="N19" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O19" s="81" t="inlineStr">
@@ -9626,18 +9626,18 @@
       </c>
       <c r="N20" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O20" s="81" t="inlineStr">
@@ -9776,18 +9776,18 @@
       </c>
       <c r="N21" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O21" s="81" t="inlineStr">
@@ -9926,18 +9926,18 @@
       </c>
       <c r="N22" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O22" s="81" t="inlineStr">
@@ -10076,18 +10076,18 @@
       </c>
       <c r="N23" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O23" s="81" t="inlineStr">
@@ -10227,39 +10227,39 @@
       </c>
       <c r="N24" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O24" s="81" t="inlineStr">
@@ -10405,39 +10405,39 @@
       </c>
       <c r="N25" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O25" s="178" t="inlineStr">
@@ -10584,12 +10584,12 @@
       </c>
       <c r="N26" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682</t>
         </is>
       </c>
       <c r="O26" s="178" t="inlineStr">
@@ -10735,12 +10735,12 @@
       </c>
       <c r="N27" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682</t>
         </is>
       </c>
       <c r="O27" s="178" t="inlineStr">
@@ -10884,39 +10884,39 @@
       </c>
       <c r="N28" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O28" s="81" t="inlineStr">
@@ -11059,39 +11059,39 @@
       </c>
       <c r="N29" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134408
-CFTS084-134409
-CFTS084-134410
-CFTS084-134411
-CFTS084-134413
-CFTS084-134561
-CFTS084-134562
-CFTS084-134566
-CFTS084-134568
-CFTS084-134644
-CFTS084-134646
-CFTS084-134701
-CFTS084-134702
-CFTS084-134703
-CFTS084-134704
-CFTS084-134705
-CFTS084-134706
-CFTS084-134707
-CFTS084-134711
-CFTS084-134712
-CFTS084-134718
-CFTS084-134724
-CFTS084-134725
-CFTS084-134727
-CFTS084-134728
-CFTS084-134729
-CFTS084-134730
-CFTS084-134731
-CFTS084-134732
-CFTS084-134733
-CFTS084-134734
-CFTS084-134735
-CFTS084-134736</t>
+          <t xml:space="preserve">CFTS084-4949379
+CFTS084-4949380
+CFTS084-4949381
+CFTS084-4949382
+CFTS084-4949384
+CFTS084-4949579
+CFTS084-4949580
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949680
+CFTS084-4949682
+CFTS084-4949746
+CFTS084-4949747
+CFTS084-4949748
+CFTS084-4949749
+CFTS084-4949750
+CFTS084-4949751
+CFTS084-4949752
+CFTS084-4949756
+CFTS084-4949757
+CFTS084-4949763
+CFTS084-4949771
+CFTS084-4949772
+CFTS084-4949774
+CFTS084-4949775
+CFTS084-4949776
+CFTS084-4949777
+CFTS084-4949778
+CFTS084-4949779
+CFTS084-4949780
+CFTS084-4949781
+CFTS084-4949782
+CFTS084-4949783</t>
         </is>
       </c>
       <c r="O29" s="178" t="inlineStr">
@@ -11236,18 +11236,18 @@
       </c>
       <c r="N30" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O30" s="81" t="inlineStr">
@@ -11392,18 +11392,18 @@
       </c>
       <c r="N31" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O31" s="178" t="inlineStr">
@@ -11546,18 +11546,18 @@
       </c>
       <c r="N32" s="178" t="inlineStr">
         <is>
-          <t xml:space="preserve">CFTS084-134565
-CFTS084-134566
-CFTS084-134568
-CFTS084-134569
-CFTS084-134570
-CFTS084-134644
-CFTS084-134645
-CFTS084-134646
-CFTS084-134714
-CFTS084-134715
-CFTS084-134716
-CFTS084-134717</t>
+          <t xml:space="preserve">CFTS084-4949587
+CFTS084-4949588
+CFTS084-4949594
+CFTS084-4949595
+CFTS084-4949596
+CFTS084-4949680
+CFTS084-4949681
+CFTS084-4949682
+CFTS084-4949759
+CFTS084-4949760
+CFTS084-4949761
+CFTS084-4949762</t>
         </is>
       </c>
       <c r="O32" s="178" t="inlineStr">

</xml_diff>

<commit_message>
feat(security): SEC-21 — apk dual-name Remarks note on 22 CertProvider TCs, security_v15
</commit_message>
<xml_diff>
--- a/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
+++ b/features/security/delivered/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
@@ -8131,7 +8131,8 @@
 Polarion: NRL-349384
 sibling axis: verification outcome; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
-apk pairing: fotaMcpuCertTestNormalFlow (apk_pairing.tsv)</t>
+apk pairing: fotaMcpuCertTestNormalFlow (apk_pairing.tsv)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -8319,7 +8320,8 @@
 channel_feasible: Y/Y
 asset: X-h — 3. PENDING: X-h log keyword
 apk pairing: fotaMcpuCertTestBrokenCert (apk_pairing.tsv)
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8508,8 @@
 sibling axis: chain trust; rule SEC-20 §2.1 (CCVR Cert Val CS.98 item 3) of SEC-04 4.2
 channel_feasible: Y/Y
 apk pairing: ecuCertTestSelfSignedChain (apk_pairing.tsv)
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -8664,7 +8667,8 @@
 Polarion: NRL-349385
 sibling axis: subject match; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/N
-apk pairing: samCertTestNormalFlow (apk_pairing.tsv)</t>
+apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8828,8 @@
 channel_feasible: Y/N
 asset: X-e — 3. PENDING: X-e wrong-subject certificate + trigger
 asset: X-h — 3. PENDING: X-h log keyword
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -8982,7 +8987,8 @@
 Polarion: NRL-349386
 sibling axis: issuer match; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/Y
-apk pairing: samCertTestNormalFlow (apk_pairing.tsv)</t>
+apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -9142,7 +9148,8 @@
 channel_feasible: Y/Y
 asset: X-e — 3. PENDING: X-e wrong-issuer certificate + trigger
 asset: X-h — 3. PENDING: X-h log keyword
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -9318,6 +9325,7 @@
 apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
 scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -9474,7 +9482,8 @@
 sibling axis: verification path; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -9647,6 +9656,7 @@
 apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
 scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -9823,6 +9833,7 @@
 apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
 scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -9999,6 +10010,7 @@
 apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
 scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -10175,6 +10187,7 @@
 apk pairing: samCertTestNormalFlow (apk_pairing.tsv)
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
 scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -11265,6 +11278,7 @@
 sibling axis: store presence; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
 conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -11457,6 +11471,7 @@
 asset: X-e — 5. PENDING: X-e valid leaf certificate + trigger
 asset: X-h — 5. PENDING: X-h log keyword
 conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -11612,7 +11627,8 @@
 asset: X-i — closed by R-SEC20 (document review; no source/build-environment asset required)
 sibling axis: client type; rule 1,4 of SEC-04 4.2
 channel_feasible: Y/Y
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -11764,7 +11780,8 @@
 asset: X-i — closed by R-SEC20 (document review; no source/build-environment asset required)
 sibling axis: client type; rule 1,4 of SEC-04 4.2
 channel_feasible: Y/Y
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -11948,6 +11965,7 @@
 sibling axis: configuration version; rule 1,2 of SEC-04 4.2
 channel_feasible: Y/Y
 conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -12137,6 +12155,7 @@
 asset: X-c — 4. PENDING: X-c NR1L production certificate + trigger
 asset: X-h — 4. PENDING: X-h log keyword
 conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)
 path per CCVR Cert Val CS.98 (RD implementation): 037 /odm/etc/cert_store = RD /vendor/odm/etc/cert_store
 term: 037 "CRL" = RD-implemented DCL file /vendor/odm/etc/cert_store/dcl.json (CCVR Cert Val CS.98)
 asset: X-e — dcl_baseline.json / dcl_revoked*.json are the pre-prepared test assets named in CCVR Cert Val CS.98 GIVEN; the steps themselves are RD-provided
@@ -12293,7 +12312,8 @@
 Polarion: NRL-349393
 sibling axis: resource consumption; rule 1,4 of SEC-04 4.2
 channel_feasible: Y/Y
-apk pairing: fotaMcpuCertVerifyStressTest (apk_pairing.tsv)</t>
+apk pairing: fotaMcpuCertVerifyStressTest (apk_pairing.tsv)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -12451,7 +12471,8 @@
 sibling axis: extension value; rule 1,3 of SEC-04 4.2
 channel_feasible: Y/N
 asset: X-e — 3. PENDING: X-e OID certificate + trigger
-asset: X-h — 3. PENDING: X-h log keyword</t>
+asset: X-h — 3. PENDING: X-h log keyword
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>
@@ -12607,7 +12628,8 @@
 channel_feasible: Y/N
 asset: X-e — 2. PENDING: X-e OID certificate + trigger
 asset: X-h — 2. PENDING: X-h log keyword
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+apk name: CCVR STEPS say CertProviderServiceManagerTest.apk; delivered file is CertProviderAndroidInstrumentalTest.apk (A-SEC-15)</t>
         </is>
       </c>
     </row>

</xml_diff>